<commit_message>
updated files after review
</commit_message>
<xml_diff>
--- a/fileOverview.xlsx
+++ b/fileOverview.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seraina/Documents/Studium/COSS/multi_currency_system/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1286CF94-DBB6-FF4B-9D46-7A2D39883704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2686565-F44D-B94C-8BA1-5EBB5A24EAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="900" windowWidth="28100" windowHeight="17240" xr2:uid="{D3400469-8806-C246-8DE7-E2184C5517B0}"/>
+    <workbookView xWindow="20" yWindow="1060" windowWidth="28100" windowHeight="17240" xr2:uid="{D3400469-8806-C246-8DE7-E2184C5517B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="60">
   <si>
     <t>Simulation script</t>
   </si>
@@ -50,18 +50,9 @@
     <t>model_data.csv</t>
   </si>
   <si>
-    <t>example_scenarios.csv</t>
-  </si>
-  <si>
-    <t>example_scenarios_randGamma_highInitLevel.csv</t>
-  </si>
-  <si>
     <t>example_scenarios.ipynb</t>
   </si>
   <si>
-    <t>example_scenarios_G_impact.csv</t>
-  </si>
-  <si>
     <t>Impact of G on stability</t>
   </si>
   <si>
@@ -86,33 +77,18 @@
     <t>example_cases_G=1_randomThresholds_highInitLevel.py</t>
   </si>
   <si>
-    <t>example_cases_G_impact.py</t>
-  </si>
-  <si>
     <t>example_cases_G=1.py</t>
   </si>
   <si>
     <t>example_cases_G=5.py</t>
   </si>
   <si>
-    <t>steepness_vs_m_c_parallel.csv</t>
-  </si>
-  <si>
     <t>eq_analysis.ipynb</t>
   </si>
   <si>
     <t>Heatmap of slopes for m vs. c</t>
   </si>
   <si>
-    <t>equilibrium_vs_s_c_likeInBsp.csv</t>
-  </si>
-  <si>
-    <t>equilibrium_vs_s_c_s=1.0.csv</t>
-  </si>
-  <si>
-    <t>equilibrium_vs_s_c_manyS.csv</t>
-  </si>
-  <si>
     <t>Analysis of mean glob param. Levels at equilibrium in dependence of s and c.</t>
   </si>
   <si>
@@ -128,12 +104,6 @@
     <t>stable_single_crisis.csv</t>
   </si>
   <si>
-    <t>recovery_time_linear.csv</t>
-  </si>
-  <si>
-    <t>random_crisis.csv</t>
-  </si>
-  <si>
     <t>recovery time in stable systems after critical jump</t>
   </si>
   <si>
@@ -149,9 +119,6 @@
     <t>random_crisis.py</t>
   </si>
   <si>
-    <t>recovery_time.py</t>
-  </si>
-  <si>
     <t>single_jump_crisis.py</t>
   </si>
   <si>
@@ -167,9 +134,6 @@
     <t>Figures in the article</t>
   </si>
   <si>
-    <t>Supplementary</t>
-  </si>
-  <si>
     <t>Fig. 4</t>
   </si>
   <si>
@@ -213,6 +177,45 @@
   </si>
   <si>
     <t>Analysis notebook</t>
+  </si>
+  <si>
+    <t>increases_crisis_a.csv</t>
+  </si>
+  <si>
+    <t>recovery_time_linear_bigS_50reps_100a_randJumpParam_s=1.5_new.csv</t>
+  </si>
+  <si>
+    <t>recovery_time_parallel.py</t>
+  </si>
+  <si>
+    <t>recovery_time_linear_bigS_50reps_100a_randJumpParam.csv</t>
+  </si>
+  <si>
+    <t>recovery time in stable systems after critical jump, one global parameter eq at 0Fig. In appendix B</t>
+  </si>
+  <si>
+    <t>Appendix B</t>
+  </si>
+  <si>
+    <t>random_crisis_sameParams.csv</t>
+  </si>
+  <si>
+    <t>example_scenarios_g=1.csv</t>
+  </si>
+  <si>
+    <t>example_scenarios_randGamma_lowInitLevel.csv</t>
+  </si>
+  <si>
+    <t>Appendix A</t>
+  </si>
+  <si>
+    <t>example_scenarios_G_impact_50reps.csv</t>
+  </si>
+  <si>
+    <t>steepness_vs_m_c_parallel_50reps.csv</t>
+  </si>
+  <si>
+    <t>equilibrium_vs_s_c_manyS_50reps_noTrading.csv</t>
   </si>
 </sst>
 </file>
@@ -297,29 +300,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -387,6 +367,29 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -401,14 +404,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FA12A10B-5B95-9040-90D7-573CA5C25961}" name="Tabelle2" displayName="Tabelle2" ref="A1:E16" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:E16" xr:uid="{FA12A10B-5B95-9040-90D7-573CA5C25961}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FA12A10B-5B95-9040-90D7-573CA5C25961}" name="Tabelle2" displayName="Tabelle2" ref="A1:E15" totalsRowShown="0" headerRowDxfId="6" dataDxfId="0">
+  <autoFilter ref="A1:E15" xr:uid="{FA12A10B-5B95-9040-90D7-573CA5C25961}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E5DB3B1E-CF24-5446-B067-FD8DC8EBFCF3}" name="Simulation script" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{FB4517EF-454C-8442-BD36-A6B94DE148EB}" name="Datafile" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{7A66DB16-53A5-A348-A8BC-69002834A7E5}" name="Analysis notebook" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{AF04D629-839A-A94E-B3BD-DF05099972E1}" name="Analysis" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{BCBBC581-F5E0-1046-90F4-D8566167444B}" name="Figures in the article" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{E5DB3B1E-CF24-5446-B067-FD8DC8EBFCF3}" name="Simulation script" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{FB4517EF-454C-8442-BD36-A6B94DE148EB}" name="Datafile" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{7A66DB16-53A5-A348-A8BC-69002834A7E5}" name="Analysis notebook" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{AF04D629-839A-A94E-B3BD-DF05099972E1}" name="Analysis" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{BCBBC581-F5E0-1046-90F4-D8566167444B}" name="Figures in the article" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -731,14 +734,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B4413E-C4C8-F04F-9ADF-447222CC2BEB}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="47.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="56.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="61.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="4" max="4" width="80.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -749,269 +752,267 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>26</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C14" s="2"/>
       <c r="D14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>47</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
-      <c r="D16" s="2" t="s">
-        <v>57</v>
-      </c>
+      <c r="D16" s="2"/>
       <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>